<commit_message>
new test Direction tetsing on stock market on HNB
</commit_message>
<xml_diff>
--- a/results_master_log.xlsx
+++ b/results_master_log.xlsx
@@ -11,7 +11,7 @@
     <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P22"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2210,8 +2210,162 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>ARDL/VECM spread test</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>9 CSE stocks + rates</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>monthly (171)</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>ARDL bounds + VECM</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>ARDL/VECM</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>long-run vs short-run</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>ARDL bounds F (banks)</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
+          <t>No long-run link (spread is I(0)); effect is short-run only; banks -, finance + but weak long-run</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>ardl_vecm_summary.md</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>spread_ardl_vecm.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Direction Step 1 baseline</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>HNB</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>80/20 chrono</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>next-day Buy/Sell/Hold</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Accuracy %</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="L24" s="2" t="n">
+        <v>43.1</v>
+      </c>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>Price+technical only: no edge, loses to persistence (43%). Honest baseline to beat.</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>step1_summary.md</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>direction_step1_baseline.py</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P22"/>
+  <autoFilter ref="A1:P24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Phase A: multi-horizon direction + return runner
</commit_message>
<xml_diff>
--- a/results_master_log.xlsx
+++ b/results_master_log.xlsx
@@ -11,7 +11,7 @@
     <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P24"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2364,8 +2364,320 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Phase A multi-horizon direction</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>HNB</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>80/20 chrono + h-bar purge</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Logistic + XGBoost</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons (1d-252d)</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Horizons beating baseline</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>0 of 9</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>majority / persistence</t>
+        </is>
+      </c>
+      <c r="M25" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="inlineStr">
+        <is>
+          <t>NO EDGE AT ANY HORIZON. Best model always below best baseline; gap widens with horizon (-3.5pp @1d -&gt; -47.1pp @1yr) because long-horizon drift makes the dumb baseline huge (maj 78% @6mo, pers 77% @1yr).</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>results/direction/multi_horizon/mh_summary.md</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>direction_multi_horizon.py; Tier-1 only; dead-zone +/-0.5%*sqrt(h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Phase A best single horizon</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>HNB</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>80/20 chrono + h-bar purge</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Logistic</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>direct, h=22d (1 month)</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Accuracy %</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="L26" s="2" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="M26" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>Best model result of the sweep (1-month Logistic 40.1%) still loses to persistence 42.1%. Logistic &gt; XGBoost at every horizon -&gt; no nonlinear structure to find.</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>mh_direction_table.csv</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>edge -2.0pp</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Return forecast</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Phase A multi-horizon return %</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>HNB</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>80/20 chrono + h-bar purge</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Ridge + XGBoost</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons (1d-252d)</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>RMSE ratio vs train-mean</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="L27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="inlineStr">
+        <is>
+          <t>Ridge beats naive-0 at 8/9 horizons BUT is only ~1% better than train-mean drift -&gt; it learned drift, NOT signal. XGBoost worse than naive everywhere (ratio 1.01-1.14).</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>mh_return_table.csv</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>train-mean is the honest null, not naive-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Return forecast</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Phase A return sign accuracy</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>HNB</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>80/20 chrono + h-bar purge</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Ridge</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>direct, sign of h-day return</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Horizons beating sign null</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>2 of 9</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>always-guess-winning-side</t>
+        </is>
+      </c>
+      <c r="M28" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N28" s="4" t="inlineStr">
+        <is>
+          <t>TRAP CHECK: 55-57% sign accuracy @1-3mo looks like the 52-58% target but 'always guess up' matches/beats it (test window drifted up 59-95%). Both 'wins' are +0.2pp = noise.</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>mh_edge_vs_horizon.png</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>up-share null added to stop false positive</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P24"/>
+  <autoFilter ref="A1:P28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
add multi-horizon direction test and tier-2 ablation for HNB
</commit_message>
<xml_diff>
--- a/results_master_log.xlsx
+++ b/results_master_log.xlsx
@@ -11,7 +11,7 @@
     <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:P31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2676,8 +2676,238 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Phase B ablation (+Tier-2)</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>HNB</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>identical rows/split/seeds, A vs B</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Logistic + XGBoost</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons, ablation</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Mean gain from Tier-2 (pp)</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="n">
+        <v>-1.1</v>
+      </c>
+      <c r="L29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
+          <t>RSI+MACD+volume add NOTHING. Mean -1.1pp, positive at only 1/9 horizons, 0/9 beat baseline. Technical indicators exhausted.</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>results/direction/phase_ablation/ablation_summary.md</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>direction_phase_ablation.py; 9 -&gt; 15 features</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Phase B feature attention check</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>HNB</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>identical rows/split/seeds</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>XGBoost importance</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Tier-2 share of importance %</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M30" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t>XGBoost spends 41% of importance on Tier-2 (macd_signal is top feature at 6/9 horizons) yet accuracy does not improve -&gt; the model USES them but they carry no signal.</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>ablation_tier2_importance.csv</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>strong evidence indicators are redundant with price</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Return forecast</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Phase B return % (+Tier-2)</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>HNB</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>identical rows/split/seeds</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Ridge + XGBoost</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>RMSE ratio vs train-mean (B)</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="n">
+        <v>0.991</v>
+      </c>
+      <c r="L31" s="2" t="n">
+        <v>0.991</v>
+      </c>
+      <c r="M31" s="3" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="N31" s="4" t="inlineStr">
+        <is>
+          <t>Tier-2 made return RMSE slightly WORSE at 9/9 horizons (ratio gain +0.000 to +0.046). Sign edge stays negative everywhere.</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>ablation_return_table.csv</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>A ratio 0.991 -&gt; B ratio 0.991-1.034</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P28"/>
+  <autoFilter ref="A1:P31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
add macro phase to direction test
</commit_message>
<xml_diff>
--- a/results_master_log.xlsx
+++ b/results_master_log.xlsx
@@ -11,7 +11,7 @@
     <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:P35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2726,7 +2726,7 @@
         </is>
       </c>
       <c r="K29" s="2" t="n">
-        <v>-1.1</v>
+        <v>-0.9</v>
       </c>
       <c r="L29" s="2" t="n">
         <v>0</v>
@@ -2738,7 +2738,7 @@
       </c>
       <c r="N29" s="4" t="inlineStr">
         <is>
-          <t>RSI+MACD+volume add NOTHING. Mean -1.1pp, positive at only 1/9 horizons, 0/9 beat baseline. Technical indicators exhausted.</t>
+          <t>RSI+MACD+volume add NOTHING. Mean -0.9pp, 0/9 beat baseline. Technical indicators exhausted.</t>
         </is>
       </c>
       <c r="O29" s="2" t="inlineStr">
@@ -2748,7 +2748,7 @@
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>direction_phase_ablation.py; 9 -&gt; 15 features</t>
+          <t>direction_phase_ablation.py; 9 -&gt; 16 features; value restated on the 4-phase run (macro availability trims early rows)</t>
         </is>
       </c>
     </row>
@@ -2906,8 +2906,314 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Phase C ablation (+macro rates)</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>HNB</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>identical rows/split/seeds, 35d publication lag</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Logistic + XGBoost</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons, ablation</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Mean gain from macro (pp)</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="L32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t>Macro rates make it WORSE and unstable: gain swings -22.3 to +10.3 pp, 0/9 beat baseline. Not weak signal - overfitting.</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>results/direction/phase_ablation/ablation_summary.md</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>direction_phase_ablation.py; 16 -&gt; 29 features; inflation/FX/M2 still uncollected</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Phase C2 diagnostic (macro changes only)</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>HNB</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>identical rows/split/seeds</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Logistic + XGBoost</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons, ablation</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Mean gain from macro d (pp)</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="L33" s="2" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="M33" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N33" s="4" t="inlineStr">
+        <is>
+          <t>DROPPING RATE LEVELS FIXES THE DAMAGE (-2.8 -&gt; +3.4 pp; 1yr 4.5% -&gt; 49.7%). Non-stationary levels were being memorised. Still 0/9 beat baseline -&gt; form was wrong AND no signal.</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>ablation_gain_table.csv</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>key methodology lesson: feed macro as changes, never levels</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Phase C feature attention check</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>HNB</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>identical rows/split/seeds</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>XGBoost importance</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Macro share of importance %</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M34" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N34" s="4" t="inlineStr">
+        <is>
+          <t>Macro importance rises 46% (1d) -&gt; 80% (1yr) while accuracy FALLS. Model fits rates as a trend proxy, not signal. tb_12m/spread/policy_rate are top features at 8/9 horizons.</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>ablation_feature_importance.csv</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>fingerprint of trending-variable overfit</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Return forecast</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Phase C return % (+macro)</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>HNB</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>identical rows/split/seeds</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Ridge + XGBoost</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>RMSE ratio vs train-mean (C)</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="L35" s="2" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="M35" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N35" s="4" t="inlineStr">
+        <is>
+          <t>Macro blows out return RMSE to 1.29-1.37x the train-mean null (A/B sat at ~0.99). Clear damage, confirms the overfit reading.</t>
+        </is>
+      </c>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>ablation_return_table.csv</t>
+        </is>
+      </c>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>worst at 2-3 month horizons</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P31"/>
+  <autoFilter ref="A1:P35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
add sector phase to direction test
</commit_message>
<xml_diff>
--- a/results_master_log.xlsx
+++ b/results_master_log.xlsx
@@ -11,7 +11,7 @@
     <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P35"/>
+  <dimension ref="A1:P39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3212,8 +3212,318 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Phase D ablation (+sector)</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>HNB</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>identical rows/split/seeds</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Logistic + XGBoost</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons, ablation</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Mean gain from sector (pp)</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="L36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N36" s="4" t="inlineStr">
+        <is>
+          <t>FIRST consistently POSITIVE step: +2.6pp mean, positive at 6/9 horizons. Built on C2 (macro changes only). But still 0/9 beat baseline.</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>results/direction/phase_ablation/ablation_summary.md</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>direction_phase_ablation.py; C2 16+7 -&gt; D 39 features; ASPI + COMB/SAMP + LOFC/LOLC/LFIN/CFIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Phase D best single horizon</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>HNB</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>identical rows/split/seeds</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Logistic + XGBoost</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>direct, h=5d (1 week)</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Edge over baseline (pp)</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="L37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N37" s="4" t="inlineStr">
+        <is>
+          <t>Closest call of the whole study: 1-week Phase D 37.3% vs baseline 37.4%. Near-parity at short horizons (1d -1.7, 1wk -0.2, 2wk -1.6) but never crosses.</t>
+        </is>
+      </c>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>ablation_gain_table.csv</t>
+        </is>
+      </c>
+      <c r="P37" s="2" t="inlineStr">
+        <is>
+          <t>not a win; single split, one stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Return forecast</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Phase D return sign edge (+sector)</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>HNB</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>identical rows/split/seeds</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Ridge + XGBoost</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>direct, sign of h-day return</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Sign edge 1wk/2wk/3wk (pp)</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>+1.7 / +1.7 / +1.1</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>always-guess-winning-side</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="N38" s="4" t="inlineStr">
+        <is>
+          <t>First POSITIVE sign edges in the study, and at 3 adjacent horizons (1-3 weeks). Tiny (~1-2pp) and one split only -&gt; flag as worth re-testing, NOT a finding.</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>ablation_return_table.csv</t>
+        </is>
+      </c>
+      <c r="P38" s="2" t="inlineStr">
+        <is>
+          <t>check on other tickers before claiming anything</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Phase D feature attention check</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>HNB</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>identical rows/split/seeds</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>XGBoost importance</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Sector share of importance %</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M39" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N39" s="4" t="inlineStr">
+        <is>
+          <t>Sector takes 34% avg (42% at 1 day, falling to 27% at 1yr) - mirror image of macro, which rises with horizon. Sector matters short, macro long, neither enough.</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>ablation_feature_importance.csv</t>
+        </is>
+      </c>
+      <c r="P39" s="2" t="inlineStr">
+        <is>
+          <t>vol_20 is top feature at 1d/1wk; d_tb3m dominates long</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P35"/>
+  <autoFilter ref="A1:P39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
add sector sweep replication test across 11 stocks
</commit_message>
<xml_diff>
--- a/results_master_log.xlsx
+++ b/results_master_log.xlsx
@@ -11,7 +11,7 @@
     <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$43</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P39"/>
+  <dimension ref="A1:P43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3522,8 +3522,320 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Sector sweep - replication test</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>11 CSE stocks (3 banks, 4 finance, 4 control)</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>80/20 chrono + h-bar purge, per stock</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Logistic + XGBoost</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons x 11 stocks</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Cells beating baseline</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>27 of 99</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>14 of 99 (Phase A)</t>
+        </is>
+      </c>
+      <c r="M40" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N40" s="4" t="inlineStr">
+        <is>
+          <t>Sector features nearly DOUBLE the win rate vs Tier-1 (14-&gt;27 of 99) but wins sit at exactly coin-flip at short horizons and collapse at long ones. No real edge.</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>results/direction/sector_sweep/sweep_summary.md</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>direction_sector_sweep.py; peer composites exclude the target stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Sector gain replication (HNB claim 3)</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>11 CSE stocks</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>identical protocol per stock</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Phase D - Phase A</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons x 11 stocks</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Mean sector gain (pp)</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="L41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N41" s="4" t="inlineStr">
+        <is>
+          <t>REPLICATES: +3.8pp mean, positive in 66/99 cells (67%), 9 of 11 stocks positive. HNB was not a fluke - sector context genuinely helps the model. Best: LFIN +13.2, SAMP +9.4, LOFC +8.2. Worst: CTC -11.0.</t>
+        </is>
+      </c>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>sweep_gain_by_ticker.csv</t>
+        </is>
+      </c>
+      <c r="P41" s="2" t="inlineStr">
+        <is>
+          <t>helping is not the same as winning</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Sector sweep significance screen</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>11 CSE stocks</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>sign test + Wilcoxon across stocks, per horizon</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>binomial sign test (H0 p=0.5)</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Best sign-test p</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L42" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M42" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N42" s="4" t="inlineStr">
+        <is>
+          <t>NOTHING SIGNIFICANT AT ANY HORIZON. Best cells (1 day, 1 week) are 6/11 stocks positive = p=0.500, exactly a coin flip. Long horizons far worse (1yr 0/11).</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>sweep_significance.csv</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>stocks share a market factor so p-values are already optimistic</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>HNB sign-edge claim retest (claim 2)</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>11 CSE stocks</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>identical protocol per stock</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Ridge + XGBoost</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>direct, sign of h-day return, 1-3 week horizons</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>Cells with positive sign edge</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>6 of 33</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>~17 of 33 (coin flip)</t>
+        </is>
+      </c>
+      <c r="M43" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N43" s="4" t="inlineStr">
+        <is>
+          <t>REFUTED. HNB's positive 1-3 week sign edge did NOT replicate - 18% vs the ~50% chance would give. It was luck. Flagged as provisional when found, now closed.</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>sweep_all_results.csv</t>
+        </is>
+      </c>
+      <c r="P43" s="2" t="inlineStr">
+        <is>
+          <t>value of naming a claim before retesting it</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P39"/>
+  <autoFilter ref="A1:P43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
add industrial production data and close the macro chapter
</commit_message>
<xml_diff>
--- a/results_master_log.xlsx
+++ b/results_master_log.xlsx
@@ -11,7 +11,7 @@
     <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$54</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P43"/>
+  <dimension ref="A1:P54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3834,8 +3834,864 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Phase E - daily USD/LKR</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>11 CSE stocks</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>80/20 chrono + h-bar purge, 2015-2026 window</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Logistic + XGBoost</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons x 11 stocks</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Mean gain from daily FX (pp)</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M44" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N44" s="4" t="inlineStr">
+        <is>
+          <t>FREQUENCY WAS NOT THE PROBLEM. Daily FX gain is exactly 0.0pp (positive in 57/99 cells = coin flip). Macro fails daily exactly as it failed monthly.</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>results/direction/daily_macro/daily_macro_summary.md</t>
+        </is>
+      </c>
+      <c r="P44" s="2" t="inlineStr">
+        <is>
+          <t>direction_daily_macro.py; new cleaned_data/usd_lkr_daily.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Phase E2 - daily global + CPI</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>11 CSE stocks</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>identical rows/split/seeds</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Logistic + XGBoost</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons x 11 stocks</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>Mean gain from global+CPI (pp)</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="n">
+        <v>-1.9</v>
+      </c>
+      <c r="L45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N45" s="4" t="inlineStr">
+        <is>
+          <t>Oil, US 10Y, DXY and inflation make it WORSE (-1.9pp), worst at long horizons (-6.0pp at 1yr). Same trending-variable overfit as Phase C.</t>
+        </is>
+      </c>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>daily_macro_gain.csv</t>
+        </is>
+      </c>
+      <c r="P45" s="2" t="inlineStr">
+        <is>
+          <t>CPI spliced across 4 base years; money supply excluded (ends 2024-08, inside test window)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Phase E significance screen</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>11 CSE stocks</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>sign test across stocks, 4 phases x 9 horizons</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>binomial sign test (H0 p=0.5)</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Combinations with p&lt;0.05</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>0 of 36</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M46" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N46" s="4" t="inlineStr">
+        <is>
+          <t>NOTHING SIGNIFICANT ANYWHERE. Best cell is 1 day (6/11 stocks, p=0.500) - exact coin flip, same as the sector sweep. Cells beating baseline: A 17, D 27, E 24, E2 25 of 99.</t>
+        </is>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>daily_macro_significance.csv</t>
+        </is>
+      </c>
+      <c r="P46" s="2" t="inlineStr">
+        <is>
+          <t>macro information source now closed at both frequencies</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Phase E feature attention check</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>11 CSE stocks</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>identical rows/split/seeds</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>XGBoost importance</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons x 11 stocks</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>New-data share of importance %</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M47" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N47" s="4" t="inlineStr">
+        <is>
+          <t>Model spends 27% of importance on the new data (FX 7%, global 11%, CPI 9%) and gains nothing - third time this fingerprint has appeared (Tier-2 41%, macro 64%, now 27%).</t>
+        </is>
+      </c>
+      <c r="O47" s="2" t="inlineStr">
+        <is>
+          <t>daily_macro_all_results.csv</t>
+        </is>
+      </c>
+      <c r="P47" s="2" t="inlineStr">
+        <is>
+          <t>using a feature is not the same as profiting from it</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Phase F - money supply (M1/M2/M2b/M4)</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>11 CSE stocks</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>80/20 chrono, sample cut at 2024-08; test 2022-03 to 2024-08</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Logistic + XGBoost</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons x 11 stocks</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>Mean gain from money supply (pp)</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="L48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M48" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N48" s="4" t="inlineStr">
+        <is>
+          <t>Money supply adds NOTHING even on a crisis-era test window (positive in 50/99 cells = exact coin flip). Window moved back so M1/M2 could be tested fairly rather than excluded.</t>
+        </is>
+      </c>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>results/direction/money_supply/money_summary.md</t>
+        </is>
+      </c>
+      <c r="P48" s="2" t="inlineStr">
+        <is>
+          <t>direction_money_supply.py; 65-day publication lag per CBSL's own note; reserve money dropped (ends 2024-02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Phase F - full classic macro set</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>11 CSE stocks</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>identical rows/split/seeds</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>Logistic + XGBoost</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons x 11 stocks</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>Mean gain money-&gt;full macro (pp)</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="L49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M49" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N49" s="4" t="inlineStr">
+        <is>
+          <t>Full classic set (money + rates + FX + inflation) = 4 of the 5 Naik-Padhi variables. Still 42/99 cells, below the money-only phase (51/99). Only industrial production remains uncollected.</t>
+        </is>
+      </c>
+      <c r="O49" s="2" t="inlineStr">
+        <is>
+          <t>money_gain.csv</t>
+        </is>
+      </c>
+      <c r="P49" s="2" t="inlineStr">
+        <is>
+          <t>closes the macro chapter apart from IIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Crisis-window effect (window sensitivity)</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>11 CSE stocks</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>2022-03 to 2024-08 vs 2024-2026</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Logistic + XGBoost</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons x 11 stocks</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>Cells beating baseline</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>43-51 of 99</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>17-27 of 99 (calm window)</t>
+        </is>
+      </c>
+      <c r="M50" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N50" s="4" t="inlineStr">
+        <is>
+          <t>IMPORTANT METHOD FINDING: moving the test window into the 2022 crisis roughly DOUBLES the win rate for ALL phases including price-only. Results are window-dependent, not model-dependent.</t>
+        </is>
+      </c>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>money_by_horizon.csv</t>
+        </is>
+      </c>
+      <c r="P50" s="2" t="inlineStr">
+        <is>
+          <t>argues for walk-forward / multi-window evaluation in the write-up</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>1-day significance - macro ruled out</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>11 CSE stocks</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>sign test across stocks, 4 phases x 9 horizons</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>binomial sign test (H0 p=0.5)</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>Cells with p&lt;0.05</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>2 of 36</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>1.8 expected by chance</t>
+        </is>
+      </c>
+      <c r="M51" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N51" s="4" t="inlineStr">
+        <is>
+          <t>Both hits are at 1 day, and the STRONGEST is Phase A (price only, 9/11, +3.9pp, p=0.033). Adding money supply SHRINKS it to +3.2pp. So it is the crisis window, not macro - and 2/36 is chance anyway.</t>
+        </is>
+      </c>
+      <c r="O51" s="2" t="inlineStr">
+        <is>
+          <t>money_significance.csv</t>
+        </is>
+      </c>
+      <c r="P51" s="2" t="inlineStr">
+        <is>
+          <t>checking the null model is what prevented a false claim</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Phase G - industrial production (IIP)</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>11 CSE stocks</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>80/20 chrono, sample 2016-2026 (IIP coverage)</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Logistic + XGBoost</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons x 11 stocks</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>Mean gain from IIP (pp)</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="n">
+        <v>-6.4</v>
+      </c>
+      <c r="L52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M52" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N52" s="4" t="inlineStr">
+        <is>
+          <t>IIP makes it WORSE (-6.4pp, positive in only 25/99 cells, 0/36 significant). It was the STRONGEST variable in the Naik-Padhi reference paper, and it still does not predict direction.</t>
+        </is>
+      </c>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>results/direction/industrial_production/iip_summary.md</t>
+        </is>
+      </c>
+      <c r="P52" s="2" t="inlineStr">
+        <is>
+          <t>direction_industrial_production.py; DCS index entered by hand, 2016-01 to 2026-05; 50-day publication lag</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Phase G - full classic macro set complete</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>11 CSE stocks</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>identical rows/split/seeds</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Logistic + XGBoost</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons x 11 stocks</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>Cells beating baseline</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>25 of 99</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>27 of 99 (no macro)</t>
+        </is>
+      </c>
+      <c r="M53" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N53" s="4" t="inlineStr">
+        <is>
+          <t>ALL FIVE Naik-Padhi macro variables now tested (IIP, money supply, T-bill rate, exchange rate, inflation). NONE beats plain price history. Macro chapter complete.</t>
+        </is>
+      </c>
+      <c r="O53" s="2" t="inlineStr">
+        <is>
+          <t>iip_gain.csv</t>
+        </is>
+      </c>
+      <c r="P53" s="2" t="inlineStr">
+        <is>
+          <t>adding all macro is WORSE than sector-only (27/99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Data quality</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>IIP seasonality guard</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Sri Lanka DCS IIP</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>monthly (125)</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>2016-01 to 2026-05</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>seasonal inspection</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>April vs March gap (pts)</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>-10 to -34</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M54" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N54" s="4" t="inlineStr">
+        <is>
+          <t>IIP is NOT seasonally adjusted - April falls 10-34 pts EVERY year (Sinhala/Tamil New Year), March always peaks. Month-on-month would be a calendar signal, so YoY-only features were used.</t>
+        </is>
+      </c>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>cleaned_data/industrial_production_monthly.csv</t>
+        </is>
+      </c>
+      <c r="P54" s="2" t="inlineStr">
+        <is>
+          <t>clean_macro_sources.py; mom column deliberately named _DO_NOT_USE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P43"/>
+  <autoFilter ref="A1:P54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
add pooled panel model, co-movement table and rule extraction
</commit_message>
<xml_diff>
--- a/results_master_log.xlsx
+++ b/results_master_log.xlsx
@@ -11,7 +11,7 @@
     <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -44,7 +44,7 @@
       <color rgb="00C00000"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -69,6 +69,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -98,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -117,6 +122,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -493,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P54"/>
+  <dimension ref="A1:P59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4690,8 +4698,400 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Correlation</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Co-movement lift table (no model)</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>7 bank/finance stocks (22,677 stock-days)</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>full panel, 15 indicators x 9 horizons</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>conditional probability + 2-proportion z</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>Median |lift| short horizons (pp)</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M55" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N55" s="4" t="inlineStr">
+        <is>
+          <t>'If indicator up, does stock go up?' answered by pure counting. Market/peer indicators give a real +6 to +10pp lift at 1d-1mo on huge samples. Macro lifts are near zero at short horizons.</t>
+        </is>
+      </c>
+      <c r="O55" s="2" t="inlineStr">
+        <is>
+          <t>results/direction/pooled_rules/comovement_table.csv</t>
+        </is>
+      </c>
+      <c r="P55" s="2" t="inlineStr">
+        <is>
+          <t>direction_pooled_and_rules.py; lift = P(up|ind up) - P(up|ind down)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Correlation</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Co-movement - long-horizon lifts are artifacts</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>7 bank/finance stocks</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>panel, |lift|&gt;=10pp cells</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>independent-window audit</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>Independent windows behind biggest lifts</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>7-24</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>hundreds needed</t>
+        </is>
+      </c>
+      <c r="M56" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N56" s="4" t="inlineStr">
+        <is>
+          <t>All 19 large lifts (T-bill -19.3, M2 +17.0, USD/LKR -15.3) sit at 3mo-1yr where only 7-24 INDEPENDENT windows exist. Overlapping windows inflate the z-test. Discard them.</t>
+        </is>
+      </c>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>comovement_table.csv</t>
+        </is>
+      </c>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>median |lift| long 4.2pp vs short 2.5pp is a sample-size illusion</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Pooled panel model (sector-wide)</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>7 bank/finance stocks pooled</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>split by DATE not row, 17,770 train rows</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>Logistic + XGBoost</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons, one model for whole sector</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>Horizons beating pooled baseline</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>2 of 9</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>majority / persistence</t>
+        </is>
+      </c>
+      <c r="M57" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N57" s="4" t="inlineStr">
+        <is>
+          <t>7x more training data (17,770 vs ~2,700 per stock). Beats the POOLED baseline at 1 day (+3.3pp) and 1 week (+2.7pp) only.</t>
+        </is>
+      </c>
+      <c r="O57" s="2" t="inlineStr">
+        <is>
+          <t>results/direction/pooled_rules/pooled_model_results.csv</t>
+        </is>
+      </c>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>direction_pooled_and_rules.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Pooled model fairness check</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>7 bank/finance stocks</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>pooled model scored vs each stock's OWN baseline</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>binomial sign test (H0 p=0.5)</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>direct, 9 horizons</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>1-day: stocks positive</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>6 of 7</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>p=0.062</t>
+        </is>
+      </c>
+      <c r="M58" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N58" s="4" t="inlineStr">
+        <is>
+          <t>STRONGEST RESULT OF THE PROJECT but still not significant. The 1-week +2.7pp was a POOLING ARTIFACT (-0.5pp vs own baselines). Only 1 day survives: median +2.5pp, p=0.062, 1 of 9 horizons, single window.</t>
+        </is>
+      </c>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>pooled_vs_own_baseline.csv</t>
+        </is>
+      </c>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>pooling stocks with different class balance weakens the majority baseline and fakes an edge</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Readable rules extracted</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>7 bank/finance stocks pooled</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>depth-3 tree, scored on unseen test set</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>Decision tree (depth 3)</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>direct, h=1/5/22</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>Best 1-day rule accuracy %</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="L59" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="M59" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N59" s="4" t="inlineStr">
+        <is>
+          <t>17 plain-English rules with out-of-sample hit rates. Best 1-day rule: calm market + flat ASPI + no big drop -&gt; Hold, 49.3% (+11.3pp). Shows WHAT the model believes, not just that it fails.</t>
+        </is>
+      </c>
+      <c r="O59" s="2" t="inlineStr">
+        <is>
+          <t>readable_rules.csv</t>
+        </is>
+      </c>
+      <c r="P59" s="2" t="inlineStr">
+        <is>
+          <t>1-month rule at 68.5% fires only 317 times - treat as noise</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P54"/>
+  <autoFilter ref="A1:P59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4710,16 +5110,16 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>RESULTS MASTER LOG — how to use</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr"/>
+      <c r="B1" s="10" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr"/>
-      <c r="B2" s="9" t="inlineStr"/>
+      <c r="B2" s="10" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4727,7 +5127,7 @@
           <t>Purpose</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
         <is>
           <t>One tidy row per reported test result, across ALL test types (forecasting, regression, event study, correlation, baseline). Filter/sort by any column.</t>
         </is>
@@ -4735,195 +5135,195 @@
     </row>
     <row r="4">
       <c r="A4" t="inlineStr"/>
-      <c r="B4" s="9" t="inlineStr"/>
+      <c r="B4" s="10" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Sequential row number</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>When the test was run (approx.)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Price forecast / Baseline / Correlation / Event study / Regression / Method study / (new types allowed)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Test / Experiment</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Short test name</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>What data (S&amp;P SL20, HNB, 10 CSE stocks, ...)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Freq</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>daily / hourly / monthly / event</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Split / Setup</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>80/20, 50/50, 40/60, walk-forward, full-sample, event-study, n specifications, ...</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Model / Method</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>ARIMA, LSTM, Hybrid, Prophet, XGBoost, GRU, TFT, OLS, event-study, ...</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>Protocol</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>one-step / multi-step / recursive / direct / n/a</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Name of the reported number (MAPE %, accuracy, interaction p, CAR, correlation, ...)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>The metric value</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>Baseline value</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>The naive / comparison value (leave '—' if not applicable)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>Beats baseline?</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>Yes / No / Tie / —  (drives the colour)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>Verdict / Key finding</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>One-line human takeaway</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>Output files</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>Where the detailed results live</t>
         </is>
@@ -4935,7 +5335,7 @@
           <t>Notes</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>Anything else (caveats, script name)</t>
         </is>
@@ -4943,15 +5343,15 @@
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
-      <c r="B22" s="9" t="inlineStr"/>
+      <c r="B22" s="10" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="inlineStr">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>RULE</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>Update this log after EVERY test run (this chat or Claude Code): add a new row to ROWS in src/build_results_log.py and re-run it, OR append a row directly in Excel. Never leave a completed test unlogged.</t>
         </is>
@@ -4963,7 +5363,7 @@
           <t>To regenerate</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>python src/build_results_log.py</t>
         </is>

</xml_diff>

<commit_message>
add walk-forward retest refuting the 1-day claim
</commit_message>
<xml_diff>
--- a/results_master_log.xlsx
+++ b/results_master_log.xlsx
@@ -11,7 +11,7 @@
     <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$62</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P59"/>
+  <dimension ref="A1:P62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -5090,8 +5090,248 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>1-day claim re-test (walk-forward)</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>7 bank/finance stocks</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>21 non-overlapping 6-month windows, expanding train</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>Logistic + XGBoost (reported separately)</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>direct, walk-forward, h=1</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>Folds with positive median edge</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>6-7 of 21</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>10.5 expected by chance</t>
+        </is>
+      </c>
+      <c r="M60" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N60" s="4" t="inlineStr">
+        <is>
+          <t>CLAIM REFUTED. Median of fold medians -1.8pp (Logistic) / -1.9pp (XGBoost), sign-test p=0.96 and 0.99. The single-split +2.5pp did not survive 21 independent windows.</t>
+        </is>
+      </c>
+      <c r="O60" s="2" t="inlineStr">
+        <is>
+          <t>results/direction/retest_1day/retest_summary.md</t>
+        </is>
+      </c>
+      <c r="P60" s="2" t="inlineStr">
+        <is>
+          <t>direction_1day_retest.py; verdict rule fixed IN ADVANCE; 1-week carried as control, also negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>1-day re-test - window regime effect</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>7 bank/finance stocks</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>21 walk-forward folds</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>Logistic + XGBoost</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>direct, h=1</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>Positive folds 2016-2020 vs 2021-2024</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>1 of 10 vs 6 of 8</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M61" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N61" s="4" t="inlineStr">
+        <is>
+          <t>Confirms the crisis-window finding a second time: folds in 2021-2024 are mostly POSITIVE, 2016-2020 mostly negative. Apparent skill is a property of the period, not the model.</t>
+        </is>
+      </c>
+      <c r="O61" s="2" t="inlineStr">
+        <is>
+          <t>retest_by_fold.csv</t>
+        </is>
+      </c>
+      <c r="P61" s="2" t="inlineStr">
+        <is>
+          <t>strong argument for walk-forward reporting in the dissertation</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>1-day re-test - per stock consistency</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>7 bank/finance stocks</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>21 walk-forward folds each</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>direct, h=1</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>Stocks positive in &gt;50% of folds</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>2 of 7</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M62" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N62" s="4" t="inlineStr">
+        <is>
+          <t>No consistency: LOFC and CFIN positive in 62% of folds, HNB in only 19%. A real edge would show across the sector, not in two names.</t>
+        </is>
+      </c>
+      <c r="O62" s="2" t="inlineStr">
+        <is>
+          <t>retest_by_stock.csv</t>
+        </is>
+      </c>
+      <c r="P62" s="2" t="inlineStr">
+        <is>
+          <t>median edge per stock ranges +4.9 (LOFC) to -4.9 (SAMP)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P59"/>
+  <autoFilter ref="A1:P62"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
add lstm and gru direction test with flat-sequence control
</commit_message>
<xml_diff>
--- a/results_master_log.xlsx
+++ b/results_master_log.xlsx
@@ -11,7 +11,7 @@
     <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$65</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P62"/>
+  <dimension ref="A1:P65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -5330,8 +5330,248 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>LSTM/GRU for direction</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>7 bank/finance stocks pooled</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>daily (30-day sequences)</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>7 walk-forward 12-month folds, 3 seeds</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>LSTM + GRU (PyTorch)</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>direct, sequence input, h=1/5/22</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>Folds positive (LSTM, h=1)</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>5 of 7</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>p=0.227</t>
+        </is>
+      </c>
+      <c r="M63" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N63" s="4" t="inlineStr">
+        <is>
+          <t>Recurrent nets do NOT beat the naive baseline at any horizon. Closes the 'did you try deep learning on direction?' question. LSTM finally applied to the direction target (project is named after it).</t>
+        </is>
+      </c>
+      <c r="O63" s="2" t="inlineStr">
+        <is>
+          <t>results/direction/lstm_gru/lstm_gru_summary.md</t>
+        </is>
+      </c>
+      <c r="P63" s="2" t="inlineStr">
+        <is>
+          <t>direction_lstm_gru.py; monthly macro excluded (flat inside a 30-day window)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Sequence vs flat control (LSTM value)</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>7 bank/finance stocks pooled</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>identical sequences, flattened for the control</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>LSTM vs Logistic on flattened sequences</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>direct, h=1/5/22</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>Median edge LSTM vs flat (pp)</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>+2.9 vs -1.7</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>Logistic(flat)</t>
+        </is>
+      </c>
+      <c r="M64" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N64" s="4" t="inlineStr">
+        <is>
+          <t>REAL NUANCE: LSTM beats the FLATTENED same data at ALL 3 horizons (1d +2.9 vs -1.7, 1wk -0.4 vs -2.1, 1mo -5.4 vs -9.9). Order of recent days carries a little signal that summary features discard - first time added complexity helped. Still not enough to reach the baseline.</t>
+        </is>
+      </c>
+      <c r="O64" s="2" t="inlineStr">
+        <is>
+          <t>lstm_gru_by_fold.csv</t>
+        </is>
+      </c>
+      <c r="P64" s="2" t="inlineStr">
+        <is>
+          <t>the flat control is what makes this interpretable</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Regime effect - THIRD confirmation</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>7 bank/finance stocks</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>7 walk-forward folds, LSTM h=1</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>Positive folds 2019-2020 vs 2021-2025</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>0 of 2 vs 5 of 5</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M65" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N65" s="4" t="inlineStr">
+        <is>
+          <t>Same window/regime pattern found for a THIRD time (after money supply and the 1-day retest). Every model looks skilled post-2021 and useless before, with identical code and features. Explains why 5/7 folds here is not convincing.</t>
+        </is>
+      </c>
+      <c r="O65" s="2" t="inlineStr">
+        <is>
+          <t>lstm_gru_by_fold.csv</t>
+        </is>
+      </c>
+      <c r="P65" s="2" t="inlineStr">
+        <is>
+          <t>strongest methodological finding of the project</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P62"/>
+  <autoFilter ref="A1:P65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
add news sentiment phase, diagnostics and full results report
</commit_message>
<xml_diff>
--- a/results_master_log.xlsx
+++ b/results_master_log.xlsx
@@ -11,7 +11,7 @@
     <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$69</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P65"/>
+  <dimension ref="A1:P69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -5570,8 +5570,320 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Phase H - news sentiment</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>7 bank/finance stocks</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>7 walk-forward 6-month folds, 2016-2022</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>Logistic + XGBoost</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>direct, h=1/5/10/22</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>Mean gain from sentiment (pp)</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M66" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N66" s="4" t="inlineStr">
+        <is>
+          <t>News sentiment does NOT improve direction. Gain positive at 2 of 4 horizons (-0.8, -0.7, +2.4, +1.6), nothing near significance (all p&gt;=0.50). No phase beats the naive baseline.</t>
+        </is>
+      </c>
+      <c r="O66" s="2" t="inlineStr">
+        <is>
+          <t>results/direction/sentiment/sentiment_summary.md</t>
+        </is>
+      </c>
+      <c r="P66" s="2" t="inlineStr">
+        <is>
+          <t>direction_phase_h_sentiment.py; 149k Dailymirror/Newsfirst articles, 9,785 market-relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Phase H - lexicon disagreement</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>Dailymirror + Newsfirst news</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>9,785 market-relevant articles 2016-2022</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>VADER vs Loughran-McDonald style</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>sentiment scoring</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>Correlation between lexicons</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="n">
+        <v>0.416</v>
+      </c>
+      <c r="L67" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M67" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N67" s="4" t="inlineStr">
+        <is>
+          <t>Two reasonable sentiment measures on the SAME articles correlate only 0.42. Direct evidence the sentiment signal is fragile, not merely weak. Running one lexicon alone would have hidden this.</t>
+        </is>
+      </c>
+      <c r="O67" s="2" t="inlineStr">
+        <is>
+          <t>sentiment_verdict.csv</t>
+        </is>
+      </c>
+      <c r="P67" s="2" t="inlineStr">
+        <is>
+          <t>finance_lexicon.py; full LM dictionary can be dropped in without code change</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Phase H - regime confound ruled out</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>7 bank/finance stocks</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>folds split calm vs crisis</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Logistic + XGBoost</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>Sentiment gain calm vs crisis (pp)</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>+0.85 vs -0.45</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M68" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N68" s="4" t="inlineStr">
+        <is>
+          <t>Expected sentiment to 'work' only in the 2022 crisis; the OPPOSITE happened (calm 9/16 folds positive, crisis 3/12). So this null is NOT a regime artifact - cleaner than the other phases.</t>
+        </is>
+      </c>
+      <c r="O68" s="2" t="inlineStr">
+        <is>
+          <t>sentiment_regime_split.csv</t>
+        </is>
+      </c>
+      <c r="P68" s="2" t="inlineStr">
+        <is>
+          <t>first phase where the regime effect did not appear</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Data quality</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>News look-ahead guard</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>Dailymirror + Newsfirst news</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>publication timestamps vs 14:30 CSE close</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>time-of-day assignment</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>Articles pushed to next trading day %</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M69" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N69" s="4" t="inlineStr">
+        <is>
+          <t>36% of articles were published AFTER the 14:30 close and were reassigned to the next trading day. Without this rule those articles report the very move being predicted and sentiment would look excellent and be worthless.</t>
+        </is>
+      </c>
+      <c r="O69" s="2" t="inlineStr">
+        <is>
+          <t>cleaned_data/news_sentiment_daily.csv</t>
+        </is>
+      </c>
+      <c r="P69" s="2" t="inlineStr">
+        <is>
+          <t>only 75 of 149,240 rows lacked a timestamp</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P65"/>
+  <autoFilter ref="A1:P69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
add hybrid arima-lstm with macro/news and paper-comparable metrics
</commit_message>
<xml_diff>
--- a/results_master_log.xlsx
+++ b/results_master_log.xlsx
@@ -11,7 +11,7 @@
     <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$85</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P80"/>
+  <dimension ref="A1:P85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -6732,8 +6732,400 @@
         </is>
       </c>
     </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Price forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid ARIMA+LSTM (Zhang 2003)</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P SL 20 + HNB</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>fixed 80/20 + 7 walk-forward folds</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>ARIMA(2,1,0) + LSTM on residuals</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>one-step-ahead, rolling ARIMA state</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>Theil U2 (fixed split)</t>
+        </is>
+      </c>
+      <c r="K81" s="2" t="n">
+        <v>1.012</v>
+      </c>
+      <c r="L81" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M81" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N81" s="4" t="inlineStr">
+        <is>
+          <t>Hybrid built properly (Y=L+N, LSTM on ARIMA residuals, 3 seeds averaged) and it does NOT beat the naive random walk. SPSL20 U2=1.012, HNB U2=1.005. Marginally WORSE than plain ARIMA on both targets.</t>
+        </is>
+      </c>
+      <c r="O81" s="2" t="inlineStr">
+        <is>
+          <t>results/hybrid_comparable/hybrid_summary.md</t>
+        </is>
+      </c>
+      <c r="P81" s="2" t="inlineStr">
+        <is>
+          <t>hybrid_arima_lstm_macro_news.py; supervisor-committed architecture, now tested</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Price forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid + macro + news (extension)</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P SL 20 + HNB</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>fixed 80/20 + 7 walk-forward folds</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>ARIMA + LSTM on residuals WITH exogenous macro/news</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>one-step-ahead</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>Folds better than naive (HNB)</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>0 of 7</t>
+        </is>
+      </c>
+      <c r="L82" s="2" t="inlineStr">
+        <is>
+          <t>naive</t>
+        </is>
+      </c>
+      <c r="M82" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N82" s="4" t="inlineStr">
+        <is>
+          <t>THE PROJECT'S EXTENSION: macro+news fed into the residual model - the part ARIMA provably cannot explain. It makes things WORSE. SPSL20 U2 1.032, HNB U2 1.011, HNB walk-forward 0/7 folds.</t>
+        </is>
+      </c>
+      <c r="O82" s="2" t="inlineStr">
+        <is>
+          <t>hybrid_walkforward_table.csv</t>
+        </is>
+      </c>
+      <c r="P82" s="2" t="inlineStr">
+        <is>
+          <t>best place to put macro if it carried information; it does not</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>Method study</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>Diebold-Mariano + Theil U added</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P SL 20 + HNB</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>fixed 80/20</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>DM test (Newey-West HAC) + Theil U2</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>forecast comparison</t>
+        </is>
+      </c>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>Models significantly better than naive</t>
+        </is>
+      </c>
+      <c r="K83" s="2" t="inlineStr">
+        <is>
+          <t>0 of 8</t>
+        </is>
+      </c>
+      <c r="L83" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M83" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N83" s="4" t="inlineStr">
+        <is>
+          <t>COMPARABILITY GAP CLOSED. Papers claim superiority with the DM test; this project had only baseline-relative edge. DM run vs naive AND vs ARIMA: ZERO models significant at p&lt;0.05. Only 1 of 8 has Theil U2&lt;1.</t>
+        </is>
+      </c>
+      <c r="O83" s="2" t="inlineStr">
+        <is>
+          <t>hybrid_fixed_split_table.csv</t>
+        </is>
+      </c>
+      <c r="P83" s="2" t="inlineStr">
+        <is>
+          <t>the standard test reviewers expect; previously missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Method study</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>R-squared on price levels is meaningless</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P SL 20 + HNB</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>fixed 80/20</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>all models incl. naive</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>R2 of the NAIVE model</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="n">
+        <v>0.9979</v>
+      </c>
+      <c r="L84" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M84" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N84" s="4" t="inlineStr">
+        <is>
+          <t>IMPORTANT FOR THE WRITE-UP: every model scores R2 0.9977-0.9980 - INCLUDING the naive random walk. Papers reporting R2~0.99 on price levels are reporting nothing. R2 on a level only measures being in the right magnitude.</t>
+        </is>
+      </c>
+      <c r="O84" s="2" t="inlineStr">
+        <is>
+          <t>hybrid_fixed_split_table.csv</t>
+        </is>
+      </c>
+      <c r="P84" s="2" t="inlineStr">
+        <is>
+          <t>direct rebuttal to a common claim in this literature</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Method study</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>Fixed split vs walk-forward disagreement</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P SL 20 + HNB</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>both protocols, same models</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>ARIMA / LSTM / Hybrid</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>one-step-ahead</t>
+        </is>
+      </c>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>ARIMA SPSL20 U2 (fixed vs WF)</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>1.005 vs 0.985</t>
+        </is>
+      </c>
+      <c r="L85" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M85" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N85" s="4" t="inlineStr">
+        <is>
+          <t>The two protocols DISAGREE: ARIMA is worse than naive on the SPSL20 fixed split (6/7 folds better in walk-forward), and the reverse pattern on HNB. Reporting only one protocol would mislead - hence both are published.</t>
+        </is>
+      </c>
+      <c r="O85" s="2" t="inlineStr">
+        <is>
+          <t>hybrid_all_results.csv</t>
+        </is>
+      </c>
+      <c r="P85" s="2" t="inlineStr">
+        <is>
+          <t>4th demonstration that the test window drives the result</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P80"/>
+  <autoFilter ref="A1:P85"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
add in-sample fitting test with random-noise control
</commit_message>
<xml_diff>
--- a/results_master_log.xlsx
+++ b/results_master_log.xlsx
@@ -11,7 +11,7 @@
     <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results log'!$A$1:$P$103</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P85"/>
+  <dimension ref="A1:P103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -7124,8 +7124,1424 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>Sector composite autocorrelation</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>BANKS/FINANCE/SECTOR composites</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>full sample</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>lag-1 autocorrelation</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>Composite vs constituent autocorr</t>
+        </is>
+      </c>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>BANKS +0.178 vs ~0.07</t>
+        </is>
+      </c>
+      <c r="L86" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M86" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N86" s="4" t="inlineStr">
+        <is>
+          <t>Averaging HELPS for banks (composite 0.178 &gt; every constituent) but FAILS for finance (0.017 - constituents have negative autocorrs that cancel). Mixing them is worse (0.078). SYSTEM DESIGN: build a BANKS index, not a banks+finance index.</t>
+        </is>
+      </c>
+      <c r="O86" s="2" t="inlineStr">
+        <is>
+          <t>results/sector_direction/autocorrelation.csv</t>
+        </is>
+      </c>
+      <c r="P86" s="2" t="inlineStr">
+        <is>
+          <t>sector_direction.py; the '6x more predictable' estimate was too strong - 1.2x on average</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>Sector direction (the product target)</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>BANKS/FINANCE/SECTOR composites</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>19 walk-forward 6-month folds</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>Logistic + XGBoost</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>direct, h=1/5/10/22, binary + 3-class</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>Configurations beating baseline</t>
+        </is>
+      </c>
+      <c r="K87" s="2" t="inlineStr">
+        <is>
+          <t>0 of 24</t>
+        </is>
+      </c>
+      <c r="L87" s="2" t="inlineStr">
+        <is>
+          <t>majority / persistence</t>
+        </is>
+      </c>
+      <c r="M87" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N87" s="4" t="inlineStr">
+        <is>
+          <t>The target the SYSTEM actually predicts, never tested before. Sector-level direction is NOT predictable on plain accuracy at any horizon or grouping. Leak scan clean.</t>
+        </is>
+      </c>
+      <c r="O87" s="2" t="inlineStr">
+        <is>
+          <t>results/sector_direction/sector_direction_summary.md</t>
+        </is>
+      </c>
+      <c r="P87" s="2" t="inlineStr">
+        <is>
+          <t>sector_direction.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>Magnitude edge on BANKS composite</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>BANKS composite</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>19 walk-forward folds, binary</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>Logistic + XGBoost</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>|return|-weighted accuracy</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>Weighted edge 1d/1wk/2wk (pp)</t>
+        </is>
+      </c>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>+10.2 / +8.1 / +11.5</t>
+        </is>
+      </c>
+      <c r="L88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M88" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N88" s="4" t="inlineStr">
+        <is>
+          <t>THIRD independent replication of the magnitude edge (after single stocks and pooled panel). Consistent across 4 horizons, 14-15 of 19 folds each, while plain accuracy edge is NEGATIVE. Product: flag big-move periods, do not emit daily direction calls.</t>
+        </is>
+      </c>
+      <c r="O88" s="2" t="inlineStr">
+        <is>
+          <t>sector_direction_all.csv</t>
+        </is>
+      </c>
+      <c r="P88" s="2" t="inlineStr">
+        <is>
+          <t>3-class magnitude figures (+34/+39pp) are INFLATED by a degenerate weighted-majority baseline - use the binary ones</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>PROBABILITY CALIBRATION (product-critical)</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>BANKS + SECTOR composites</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>19 walk-forward folds, calibrator fitted inside training window only</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>Logistic/XGBoost x raw/Platt/isotonic</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>binary, h=5/10/22</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>Configurations usable (skill&gt;0 &amp; ECE&lt;0.10)</t>
+        </is>
+      </c>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t>0 of 36</t>
+        </is>
+      </c>
+      <c r="L89" s="2" t="inlineStr">
+        <is>
+          <t>climatology (base rate)</t>
+        </is>
+      </c>
+      <c r="M89" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N89" s="4" t="inlineStr">
+        <is>
+          <t>THE DASHBOARD CANNOT SHOW A MODEL CONFIDENCE NUMBER. Every Brier skill score is NEGATIVE; AUC 0.41-0.56 = coin flip. Calibration cannot fix a model that cannot rank.</t>
+        </is>
+      </c>
+      <c r="O89" s="2" t="inlineStr">
+        <is>
+          <t>results/sector_calibration/calibration_summary.md</t>
+        </is>
+      </c>
+      <c r="P89" s="2" t="inlineStr">
+        <is>
+          <t>sector_calibration.py; sklearn 1.9 removed cv='prefit', FrozenEstimator required</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>Calibration removes error by removing information</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>BANKS + SECTOR composites</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>19 walk-forward folds</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>Platt vs raw probabilities</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>prob_std Platt vs raw</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t>0.012-0.054 vs 0.164-0.232</t>
+        </is>
+      </c>
+      <c r="L90" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M90" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N90" s="4" t="inlineStr">
+        <is>
+          <t>Platt roughly HALVES calibration error by collapsing the forecast to near-constant. A model that says '54%' every day is perfectly calibrated and useless - no resolution. Calibration alone is not evidence of a usable forecast.</t>
+        </is>
+      </c>
+      <c r="O90" s="2" t="inlineStr">
+        <is>
+          <t>calibration_all_folds.csv</t>
+        </is>
+      </c>
+      <c r="P90" s="2" t="inlineStr">
+        <is>
+          <t>product answer: replace model confidence with a realised track record</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>News isolated - macro removed</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>BANKS composite + S&amp;P SL 20</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>6 walk-forward folds, 2016-2022 (news window)</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>Logistic + XGBoost</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>direct, h=1/5/10, P vs P+N</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>Horizons where news helps</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr">
+        <is>
+          <t>0 of 6</t>
+        </is>
+      </c>
+      <c r="L91" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M91" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N91" s="4" t="inlineStr">
+        <is>
+          <t>CLEAN ISOLATION TEST. In Phase H news competed with ~30 other columns incl. macro, which Phase C showed can actively hurt. Stripped back to price+news only: news gain -1.25 to +2.60pp, nothing significant. Macro was NOT masking news.</t>
+        </is>
+      </c>
+      <c r="O91" s="2" t="inlineStr">
+        <is>
+          <t>results/price_news_hybrid/news_gain.csv</t>
+        </is>
+      </c>
+      <c r="P91" s="2" t="inlineStr">
+        <is>
+          <t>price_news_hybrid.py; window 2016-2022 not comparable to other phases</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Price forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid + news, no macro</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>BANKS composite + S&amp;P SL 20</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>6 walk-forward folds</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>naive / ARIMA(2,1,0) / Hybrid / Hybrid+News</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>one-step-ahead</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>Theil U2 (Hybrid+News, BANKS)</t>
+        </is>
+      </c>
+      <c r="K92" s="2" t="n">
+        <v>1.0003</v>
+      </c>
+      <c r="L92" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M92" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N92" s="4" t="inlineStr">
+        <is>
+          <t>Adding news to the hybrid makes it WORSE on both targets (BANKS 0.989-&gt;1.000, SPSL20 0.987-&gt;1.017). Plain ARIMA is the best model in the table and even it is not significant (DM p=0.30/0.46). Simplest wins again.</t>
+        </is>
+      </c>
+      <c r="O92" s="2" t="inlineStr">
+        <is>
+          <t>results/price_news_hybrid/price_summary.csv</t>
+        </is>
+      </c>
+      <c r="P92" s="2" t="inlineStr">
+        <is>
+          <t>supports cutting BOTH the news and hybrid stages from the production system</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>Data quality</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>LEAK #4 - SPSL20 calendar vs ASPI (again)</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P SL 20</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>feature vs same-day and next-day return</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>correlation audit</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>leak detection</t>
+        </is>
+      </c>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>corr with next-day vs same-day</t>
+        </is>
+      </c>
+      <c r="K93" s="2" t="n">
+        <v>0.871</v>
+      </c>
+      <c r="L93" s="2" t="n">
+        <v>0.227</v>
+      </c>
+      <c r="M93" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N93" s="4" t="inlineStr">
+        <is>
+          <t>The 'clean' SPSL20 file DELETED every flat day, misaligning it against ASPI (352 of 1505 rows drop). Removing .ffill() was NOT enough. Faked 82.8% accuracy / +20.7pp edge; a trivial 'copy sign of ASPI' rule scored 84.3%. Fixed by using the ASPI-calendar SPSL20 file AND dropping ASPI features for index targets.</t>
+        </is>
+      </c>
+      <c r="O93" s="2" t="inlineStr">
+        <is>
+          <t>results/price_news_hybrid/leak_scan.csv</t>
+        </is>
+      </c>
+      <c r="P93" s="2" t="inlineStr">
+        <is>
+          <t>corrected result: 56.8% accuracy, -5.5pp edge</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Method study</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>Leak guard now HALTS the run</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>all targets</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>every feature set</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>automated leak scan</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>guard</t>
+        </is>
+      </c>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>Runs aborted on leak detection</t>
+        </is>
+      </c>
+      <c r="K94" s="2" t="inlineStr">
+        <is>
+          <t>1 of 1</t>
+        </is>
+      </c>
+      <c r="L94" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M94" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N94" s="4" t="inlineStr">
+        <is>
+          <t>The guard previously only wrote a CSV and the run continued, reporting a fake +20.7pp edge while the summary line claimed 'clean'. A guard that does not stop the run is not a guard. Now raises SystemExit.</t>
+        </is>
+      </c>
+      <c r="O94" s="2" t="inlineStr">
+        <is>
+          <t>price_news_hybrid.py</t>
+        </is>
+      </c>
+      <c r="P94" s="2" t="inlineStr">
+        <is>
+          <t>4th leak caught in this project; all four flattered the model</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>Late fusion (one model per source)</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>BANKS composite + HNB</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>6 walk-forward folds, chronological base/meta split</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>XGBoost bases + Logistic meta-learner</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t>stacking, h=1/5/10</t>
+        </is>
+      </c>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>Configurations beating baseline</t>
+        </is>
+      </c>
+      <c r="K95" s="2" t="inlineStr">
+        <is>
+          <t>0 of 6</t>
+        </is>
+      </c>
+      <c r="L95" s="2" t="inlineStr">
+        <is>
+          <t>majority / persistence</t>
+        </is>
+      </c>
+      <c r="M95" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N95" s="4" t="inlineStr">
+        <is>
+          <t>ARCHITECTURE WAS NOT THE CONSTRAINT. Separate models for price/news/macro combined by a meta-learner: 0/6 beat the baseline. Late fusion IS less bad than early fusion (better in 5/6) but beats it significantly in only 1/6 = chance.</t>
+        </is>
+      </c>
+      <c r="O95" s="2" t="inlineStr">
+        <is>
+          <t>results/late_fusion/late_fusion_summary.md</t>
+        </is>
+      </c>
+      <c r="P95" s="2" t="inlineStr">
+        <is>
+          <t>late_fusion_stacking.py; meta-learner trained on OUT-OF-FOLD base predictions</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>Meta-learner weight allocation</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>BANKS composite + HNB</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>6 walk-forward folds</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>Logistic meta-learner on 3 base models</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>stacking</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>Median weight share price/news/macro</t>
+        </is>
+      </c>
+      <c r="K96" s="2" t="inlineStr">
+        <is>
+          <t>29% / 38% / 33%</t>
+        </is>
+      </c>
+      <c r="L96" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M96" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N96" s="4" t="inlineStr">
+        <is>
+          <t>CLEANEST VERSION OF THE CENTRAL FINDING. A model free to weight the three sources however it likes splits ~1/3 each and leans MOST on news. If price carried signal and news did not, it would load onto price. Even allocation = nothing to prefer.</t>
+        </is>
+      </c>
+      <c r="O96" s="2" t="inlineStr">
+        <is>
+          <t>results/late_fusion/meta_weights_summary.csv</t>
+        </is>
+      </c>
+      <c r="P96" s="2" t="inlineStr">
+        <is>
+          <t>resolves the ambiguous early-fusion result (high importance, zero gain)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Method study</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>Early vs late fusion ruled out as explanation</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>BANKS composite + HNB</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>identical folds, both architectures</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>early (concatenated) vs late (stacked)</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr">
+        <is>
+          <t>direction</t>
+        </is>
+      </c>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>Late beats early significantly</t>
+        </is>
+      </c>
+      <c r="K97" s="2" t="inlineStr">
+        <is>
+          <t>1 of 6</t>
+        </is>
+      </c>
+      <c r="L97" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M97" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N97" s="4" t="inlineStr">
+        <is>
+          <t>Rules out one candidate explanation for why published papers report gains: 'early fusion drowned the weak signals'. Giving news and macro dedicated models surfaces nothing. Still open: missing naive baselines, no publication lag, single favourable split, decomposition hybrids.</t>
+        </is>
+      </c>
+      <c r="O97" s="2" t="inlineStr">
+        <is>
+          <t>late_fusion_folds.csv</t>
+        </is>
+      </c>
+      <c r="P97" s="2" t="inlineStr">
+        <is>
+          <t>late_fusion_stacking.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Method study</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>Reproduce-then-break ladder</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P SL 20 + BANKS composite</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>L0 paper-style -&gt; L3 walk-forward, one guard at a time</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>Ridge + XGBoost (best reported)</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>next-day price</t>
+        </is>
+      </c>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>L0 'macro improvement' %</t>
+        </is>
+      </c>
+      <c r="K98" s="2" t="inlineStr">
+        <is>
+          <t>+0.17 / -0.04</t>
+        </is>
+      </c>
+      <c r="L98" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M98" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N98" s="4" t="inlineStr">
+        <is>
+          <t>REPRODUCTION FAILED - and that is the finding. Removing the publication lag, leaking the scaler and using a single split move the number by FRACTIONS OF A PERCENT. These three shortcuts are NOT the mechanism behind published macro gains.</t>
+        </is>
+      </c>
+      <c r="O98" s="2" t="inlineStr">
+        <is>
+          <t>results/reproduce_then_break/ladder_summary.md</t>
+        </is>
+      </c>
+      <c r="P98" s="2" t="inlineStr">
+        <is>
+          <t>reproduce_then_break.py; hypothesis was wrong, reported as such</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>Method study</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>The likely real mechanism: no naive baseline</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P SL 20 + BANKS composite</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>all ladder levels</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>all configs incl. naive</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
+          <t>next-day price</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>R2 across every level</t>
+        </is>
+      </c>
+      <c r="K99" s="2" t="n">
+        <v>0.998</v>
+      </c>
+      <c r="L99" s="2" t="n">
+        <v>0.9979</v>
+      </c>
+      <c r="M99" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N99" s="4" t="inlineStr">
+        <is>
+          <t>R2 is 0.9978-0.9984 at EVERY level for EVERY config - and naive scores 0.9979. A paper running this exact setup would truthfully report 'R2=0.998, MAPE=0.83%, outperforms benchmark'. The gain is model-vs-weaker-model, reported with metrics that cannot distinguish either from a random walk.</t>
+        </is>
+      </c>
+      <c r="O99" s="2" t="inlineStr">
+        <is>
+          <t>ladder_summary.csv</t>
+        </is>
+      </c>
+      <c r="P99" s="2" t="inlineStr">
+        <is>
+          <t>DM p = 0.48-0.86 throughout; nothing significant</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Method study</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>Single split is the shortcut that matters most</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P SL 20 + BANKS composite</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>L0-L2 single split vs L3 walk-forward</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>Ridge + XGBoost</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr">
+        <is>
+          <t>next-day price</t>
+        </is>
+      </c>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>MAPE(macro)/MAPE(naive)</t>
+        </is>
+      </c>
+      <c r="K100" s="2" t="inlineStr">
+        <is>
+          <t>0.96-0.98 -&gt; 1.027</t>
+        </is>
+      </c>
+      <c r="L100" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="M100" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N100" s="4" t="inlineStr">
+        <is>
+          <t>Under single-split levels price+macro sits BELOW naive (0.964-0.980); under walk-forward it crosses ABOVE 1.0 on both targets. Of the three shortcuts tested, the single split changes the conclusion; the other two do not. 4th confirmation of the window effect.</t>
+        </is>
+      </c>
+      <c r="O100" s="2" t="inlineStr">
+        <is>
+          <t>ladder_all.csv</t>
+        </is>
+      </c>
+      <c r="P100" s="2" t="inlineStr">
+        <is>
+          <t>argues for walk-forward as the default reporting protocol</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>Method study</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>DECOMPOSITION LEAK - the mechanism found</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P SL 20 + BANKS composite</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>fixed 80/20, identical model/data, only pipeline ORDER differs</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>wavelet(db4,3) + CEEMDAN -&gt; Ridge/XGBoost</t>
+        </is>
+      </c>
+      <c r="I101" s="2" t="inlineStr">
+        <is>
+          <t>one-step-ahead price</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>Improvement over naive: leaky vs honest</t>
+        </is>
+      </c>
+      <c r="K101" s="2" t="inlineStr">
+        <is>
+          <t>+19.2% vs -6.9%</t>
+        </is>
+      </c>
+      <c r="L101" s="2" t="inlineStr">
+        <is>
+          <t>naive</t>
+        </is>
+      </c>
+      <c r="M101" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N101" s="4" t="inlineStr">
+        <is>
+          <t>★ THE MECHANISM. Decomposing the FULL series BEFORE splitting creates a 13-26pp improvement out of nothing. Wavelet/CEEMDAN are GLOBAL transforms: component values at time t are computed from the whole series, so training components carry test-period information and test components were built from their own future.</t>
+        </is>
+      </c>
+      <c r="O101" s="2" t="inlineStr">
+        <is>
+          <t>results/decomposition_leak/decomposition_summary.md</t>
+        </is>
+      </c>
+      <c r="P101" s="2" t="inlineStr">
+        <is>
+          <t>decomposition_leak_test.py; explains the gap between published hybrid results and this project</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Method study</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>Leaky decomposition is highly significant</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P SL 20 + BANKS composite</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>fixed 80/20</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>wavelet + CEEMDAN, leaky pipeline</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t>one-step-ahead price</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>DM p vs naive (4 configs)</t>
+        </is>
+      </c>
+      <c r="K102" s="2" t="inlineStr">
+        <is>
+          <t>0.0000-0.0199</t>
+        </is>
+      </c>
+      <c r="L102" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M102" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N102" s="4" t="inlineStr">
+        <is>
+          <t>ALL FOUR leaky configurations beat naive significantly (Theil U2 0.794-0.871, DM p&lt;0.02, two at p&lt;0.0001). These are exactly the numbers decomposition-hybrid papers report.</t>
+        </is>
+      </c>
+      <c r="O102" s="2" t="inlineStr">
+        <is>
+          <t>decomposition_results.csv</t>
+        </is>
+      </c>
+      <c r="P102" s="2" t="inlineStr">
+        <is>
+          <t>the result is real as computed - it is the pipeline that is wrong</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>Method study</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>Honest decomposition loses to naive</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P SL 20 + BANKS composite</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>fixed 80/20, decompose only series[:t] at each t</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>wavelet + CEEMDAN, honest pipeline</t>
+        </is>
+      </c>
+      <c r="I103" s="2" t="inlineStr">
+        <is>
+          <t>one-step-ahead price</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t>Theil U2 (4 configs)</t>
+        </is>
+      </c>
+      <c r="K103" s="2" t="inlineStr">
+        <is>
+          <t>1.008-1.028</t>
+        </is>
+      </c>
+      <c r="L103" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M103" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N103" s="4" t="inlineStr">
+        <is>
+          <t>Same models, same data, decomposition restricted to past data only: ALL FOUR configs are WORSE than a random walk and none significant (DM p 0.35-0.84). The decomposition advantage does not survive an honest pipeline.</t>
+        </is>
+      </c>
+      <c r="O103" s="2" t="inlineStr">
+        <is>
+          <t>decomposition_results.csv</t>
+        </is>
+      </c>
+      <c r="P103" s="2" t="inlineStr">
+        <is>
+          <t>honest CEEMDAN re-decomposes every 3rd point for runtime; wavelet every point</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P85"/>
+  <autoFilter ref="A1:P103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>